<commit_message>
Changes made for Bolivia db
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/daysofweek_list.xlsx
+++ b/mosip_master/xlsx/daysofweek_list.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8555"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="daysofweek_list" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="32">
   <si>
     <t>code</t>
   </si>
@@ -77,7 +77,13 @@
     <t>t</t>
   </si>
   <si>
-    <t>System</t>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>MON</t>
+  </si>
+  <si>
+    <t>masterdata-220005</t>
   </si>
   <si>
     <t>TUE</t>
@@ -95,33 +101,15 @@
     <t>SAT</t>
   </si>
   <si>
-    <t>रवि</t>
-  </si>
-  <si>
-    <t>hin</t>
-  </si>
-  <si>
-    <t>मंगल</t>
-  </si>
-  <si>
-    <t>बुध</t>
-  </si>
-  <si>
-    <t>इकट्ठा करना</t>
-  </si>
-  <si>
-    <t>शुक्र</t>
-  </si>
-  <si>
-    <t>बैठा</t>
-  </si>
-  <si>
     <t>DOM</t>
   </si>
   <si>
     <t>es</t>
   </si>
   <si>
+    <t>LUN</t>
+  </si>
+  <si>
     <t>MAR</t>
   </si>
   <si>
@@ -135,47 +123,18 @@
   </si>
   <si>
     <t>Sáb</t>
-  </si>
-  <si>
-    <t>DIM</t>
-  </si>
-  <si>
-    <t>fra</t>
-  </si>
-  <si>
-    <t>MER</t>
-  </si>
-  <si>
-    <t>JEU</t>
-  </si>
-  <si>
-    <t>VEN</t>
-  </si>
-  <si>
-    <t>SAM</t>
-  </si>
-  <si>
-    <t>MON</t>
-  </si>
-  <si>
-    <t>masterdata-220005</t>
-  </si>
-  <si>
-    <t>सोमवार</t>
-  </si>
-  <si>
-    <t>LUN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="180" formatCode="dd/mm/yyyy\ hh:mm"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -780,11 +739,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="47" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1322,6 +1284,10 @@
   <sheetPr/>
   <dimension ref="A1:L29"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="8" max="8" width="16.7777777777778"/>
+    <col min="10" max="10" width="27.1111111111111" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
@@ -1384,7 +1350,7 @@
         <v>16</v>
       </c>
       <c r="H2" s="1">
-        <v>45526.60499971</v>
+        <v>45667.2624296121</v>
       </c>
       <c r="K2" t="s">
         <v>13</v>
@@ -1392,13 +1358,13 @@
     </row>
     <row r="3" spans="1:11">
       <c r="A3">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B3" t="s">
         <v>17</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D3" t="s">
         <v>15</v>
@@ -1413,7 +1379,13 @@
         <v>16</v>
       </c>
       <c r="H3" s="1">
-        <v>45526.60499971</v>
+        <v>45667.2624296121</v>
+      </c>
+      <c r="I3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" s="2">
+        <v>45663.2521643518</v>
       </c>
       <c r="K3" t="s">
         <v>13</v>
@@ -1421,13 +1393,13 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D4" t="s">
         <v>15</v>
@@ -1442,7 +1414,7 @@
         <v>16</v>
       </c>
       <c r="H4" s="1">
-        <v>45526.60499971</v>
+        <v>45667.2624296121</v>
       </c>
       <c r="K4" t="s">
         <v>13</v>
@@ -1450,13 +1422,13 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" t="s">
         <v>15</v>
@@ -1471,21 +1443,23 @@
         <v>16</v>
       </c>
       <c r="H5" s="1">
-        <v>45526.60499971</v>
-      </c>
+        <v>45667.2624296121</v>
+      </c>
+      <c r="I5"/>
+      <c r="J5"/>
       <c r="K5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D6" t="s">
         <v>15</v>
@@ -1500,7 +1474,7 @@
         <v>16</v>
       </c>
       <c r="H6" s="1">
-        <v>45526.60499971</v>
+        <v>45667.2624296121</v>
       </c>
       <c r="K6" t="s">
         <v>13</v>
@@ -1508,16 +1482,16 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E7" t="s">
         <v>14</v>
@@ -1529,7 +1503,7 @@
         <v>16</v>
       </c>
       <c r="H7" s="1">
-        <v>45526.60499971</v>
+        <v>45667.2624296121</v>
       </c>
       <c r="K7" t="s">
         <v>13</v>
@@ -1537,19 +1511,19 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D8" t="s">
         <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F8" t="s">
         <v>15</v>
@@ -1558,7 +1532,7 @@
         <v>16</v>
       </c>
       <c r="H8" s="1">
-        <v>45526.60499971</v>
+        <v>45667.2624296121</v>
       </c>
       <c r="K8" t="s">
         <v>13</v>
@@ -1566,19 +1540,19 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B9" t="s">
         <v>24</v>
       </c>
       <c r="C9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F9" t="s">
         <v>15</v>
@@ -1587,27 +1561,29 @@
         <v>16</v>
       </c>
       <c r="H9" s="1">
-        <v>45526.60499971</v>
-      </c>
+        <v>45667.2624296121</v>
+      </c>
+      <c r="I9"/>
+      <c r="J9"/>
       <c r="K9" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" t="s">
         <v>25</v>
-      </c>
-      <c r="C10">
-        <v>4</v>
-      </c>
-      <c r="D10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" t="s">
-        <v>23</v>
       </c>
       <c r="F10" t="s">
         <v>15</v>
@@ -1616,7 +1592,13 @@
         <v>16</v>
       </c>
       <c r="H10" s="1">
-        <v>45526.60499971</v>
+        <v>45667.2624296121</v>
+      </c>
+      <c r="I10" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="1">
+        <v>45663.2521686458</v>
       </c>
       <c r="K10" t="s">
         <v>13</v>
@@ -1624,19 +1606,19 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D11" t="s">
         <v>15</v>
       </c>
       <c r="E11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F11" t="s">
         <v>15</v>
@@ -1645,7 +1627,7 @@
         <v>16</v>
       </c>
       <c r="H11" s="1">
-        <v>45526.60499971</v>
+        <v>45667.2624296121</v>
       </c>
       <c r="K11" t="s">
         <v>13</v>
@@ -1653,19 +1635,19 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C12">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D12" t="s">
         <v>15</v>
       </c>
       <c r="E12" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F12" t="s">
         <v>15</v>
@@ -1674,7 +1656,7 @@
         <v>16</v>
       </c>
       <c r="H12" s="1">
-        <v>45526.60499971</v>
+        <v>45667.2624296121</v>
       </c>
       <c r="K12" t="s">
         <v>13</v>
@@ -1682,19 +1664,19 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C13">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D13" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F13" t="s">
         <v>15</v>
@@ -1702,8 +1684,8 @@
       <c r="G13" t="s">
         <v>16</v>
       </c>
-      <c r="H13" s="1">
-        <v>45526.60499971</v>
+      <c r="H13" s="2">
+        <v>45667.2624305556</v>
       </c>
       <c r="K13" t="s">
         <v>13</v>
@@ -1711,19 +1693,19 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D14" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E14" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F14" t="s">
         <v>15</v>
@@ -1732,7 +1714,7 @@
         <v>16</v>
       </c>
       <c r="H14" s="1">
-        <v>45526.60499971</v>
+        <v>45667.2624296121</v>
       </c>
       <c r="K14" t="s">
         <v>13</v>
@@ -1740,19 +1722,19 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B15" t="s">
         <v>31</v>
       </c>
       <c r="C15">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D15" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E15" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F15" t="s">
         <v>15</v>
@@ -1761,441 +1743,63 @@
         <v>16</v>
       </c>
       <c r="H15" s="1">
-        <v>45526.60499971</v>
-      </c>
+        <v>45667.2624296121</v>
+      </c>
+      <c r="I15"/>
+      <c r="J15"/>
       <c r="K15" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
-      <c r="A16">
-        <v>104</v>
-      </c>
-      <c r="B16" t="s">
-        <v>32</v>
-      </c>
-      <c r="C16">
-        <v>4</v>
-      </c>
-      <c r="D16" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16" t="s">
-        <v>30</v>
-      </c>
-      <c r="F16" t="s">
-        <v>15</v>
-      </c>
-      <c r="G16" t="s">
-        <v>16</v>
-      </c>
-      <c r="H16" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="K16" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11">
-      <c r="A17">
-        <v>105</v>
-      </c>
-      <c r="B17" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17">
-        <v>5</v>
-      </c>
-      <c r="D17" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17" t="s">
-        <v>30</v>
-      </c>
-      <c r="F17" t="s">
-        <v>15</v>
-      </c>
-      <c r="G17" t="s">
-        <v>16</v>
-      </c>
-      <c r="H17" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="K17" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
-      <c r="A18">
-        <v>106</v>
-      </c>
-      <c r="B18" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18">
-        <v>6</v>
-      </c>
-      <c r="D18" t="s">
-        <v>15</v>
-      </c>
-      <c r="E18" t="s">
-        <v>30</v>
-      </c>
-      <c r="F18" t="s">
-        <v>15</v>
-      </c>
-      <c r="G18" t="s">
-        <v>16</v>
-      </c>
-      <c r="H18" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="K18" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11">
-      <c r="A19">
-        <v>107</v>
-      </c>
-      <c r="B19" t="s">
-        <v>35</v>
-      </c>
-      <c r="C19">
-        <v>7</v>
-      </c>
-      <c r="D19" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" t="s">
-        <v>30</v>
-      </c>
-      <c r="F19" t="s">
-        <v>15</v>
-      </c>
-      <c r="G19" t="s">
-        <v>16</v>
-      </c>
-      <c r="H19" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="K19" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11">
-      <c r="A20">
-        <v>101</v>
-      </c>
-      <c r="B20" t="s">
-        <v>36</v>
-      </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-      <c r="D20" t="s">
-        <v>13</v>
-      </c>
-      <c r="E20" t="s">
-        <v>37</v>
-      </c>
-      <c r="F20" t="s">
-        <v>15</v>
-      </c>
-      <c r="G20" t="s">
-        <v>16</v>
-      </c>
-      <c r="H20" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="K20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11">
-      <c r="A21">
-        <v>103</v>
-      </c>
-      <c r="B21" t="s">
-        <v>31</v>
-      </c>
-      <c r="C21">
-        <v>3</v>
-      </c>
-      <c r="D21" t="s">
-        <v>15</v>
-      </c>
-      <c r="E21" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21" t="s">
-        <v>15</v>
-      </c>
-      <c r="G21" t="s">
-        <v>16</v>
-      </c>
-      <c r="H21" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="K21" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11">
-      <c r="A22">
-        <v>104</v>
-      </c>
-      <c r="B22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C22">
-        <v>4</v>
-      </c>
-      <c r="D22" t="s">
-        <v>15</v>
-      </c>
-      <c r="E22" t="s">
-        <v>37</v>
-      </c>
-      <c r="F22" t="s">
-        <v>15</v>
-      </c>
-      <c r="G22" t="s">
-        <v>16</v>
-      </c>
-      <c r="H22" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="K22" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11">
-      <c r="A23">
-        <v>105</v>
-      </c>
-      <c r="B23" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23">
-        <v>5</v>
-      </c>
-      <c r="D23" t="s">
-        <v>15</v>
-      </c>
-      <c r="E23" t="s">
-        <v>37</v>
-      </c>
-      <c r="F23" t="s">
-        <v>15</v>
-      </c>
-      <c r="G23" t="s">
-        <v>16</v>
-      </c>
-      <c r="H23" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="K23" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11">
-      <c r="A24">
-        <v>106</v>
-      </c>
-      <c r="B24" t="s">
-        <v>40</v>
-      </c>
-      <c r="C24">
-        <v>6</v>
-      </c>
-      <c r="D24" t="s">
-        <v>15</v>
-      </c>
-      <c r="E24" t="s">
-        <v>37</v>
-      </c>
-      <c r="F24" t="s">
-        <v>15</v>
-      </c>
-      <c r="G24" t="s">
-        <v>16</v>
-      </c>
-      <c r="H24" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="K24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11">
-      <c r="A25">
-        <v>107</v>
-      </c>
-      <c r="B25" t="s">
-        <v>41</v>
-      </c>
-      <c r="C25">
-        <v>7</v>
-      </c>
-      <c r="D25" t="s">
-        <v>13</v>
-      </c>
-      <c r="E25" t="s">
-        <v>37</v>
-      </c>
-      <c r="F25" t="s">
-        <v>15</v>
-      </c>
-      <c r="G25" t="s">
-        <v>16</v>
-      </c>
-      <c r="H25" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="K25" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11">
-      <c r="A26">
-        <v>102</v>
-      </c>
-      <c r="B26" t="s">
-        <v>42</v>
-      </c>
-      <c r="C26">
-        <v>2</v>
-      </c>
-      <c r="D26" t="s">
-        <v>15</v>
-      </c>
-      <c r="E26" t="s">
-        <v>14</v>
-      </c>
-      <c r="F26" t="s">
-        <v>15</v>
-      </c>
-      <c r="G26" t="s">
-        <v>16</v>
-      </c>
-      <c r="H26" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="I26" t="s">
-        <v>43</v>
-      </c>
-      <c r="J26" s="1">
-        <v>45663.2521686467</v>
-      </c>
-      <c r="K26" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11">
-      <c r="A27">
-        <v>102</v>
-      </c>
-      <c r="B27" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27">
-        <v>2</v>
-      </c>
-      <c r="D27" t="s">
-        <v>15</v>
-      </c>
-      <c r="E27" t="s">
-        <v>23</v>
-      </c>
-      <c r="F27" t="s">
-        <v>15</v>
-      </c>
-      <c r="G27" t="s">
-        <v>16</v>
-      </c>
-      <c r="H27" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="I27" t="s">
-        <v>43</v>
-      </c>
-      <c r="J27" s="1">
-        <v>45663.2521686467</v>
-      </c>
-      <c r="K27" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11">
-      <c r="A28">
-        <v>102</v>
-      </c>
-      <c r="B28" t="s">
-        <v>45</v>
-      </c>
-      <c r="C28">
-        <v>2</v>
-      </c>
-      <c r="D28" t="s">
-        <v>15</v>
-      </c>
-      <c r="E28" t="s">
-        <v>30</v>
-      </c>
-      <c r="F28" t="s">
-        <v>15</v>
-      </c>
-      <c r="G28" t="s">
-        <v>16</v>
-      </c>
-      <c r="H28" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="I28" t="s">
-        <v>43</v>
-      </c>
-      <c r="J28" s="1">
-        <v>45663.2521686467</v>
-      </c>
-      <c r="K28" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11">
-      <c r="A29">
-        <v>102</v>
-      </c>
-      <c r="B29" t="s">
-        <v>45</v>
-      </c>
-      <c r="C29">
-        <v>2</v>
-      </c>
-      <c r="D29" t="s">
-        <v>15</v>
-      </c>
-      <c r="E29" t="s">
-        <v>37</v>
-      </c>
-      <c r="F29" t="s">
-        <v>15</v>
-      </c>
-      <c r="G29" t="s">
-        <v>16</v>
-      </c>
-      <c r="H29" s="1">
-        <v>45526.60499971</v>
-      </c>
-      <c r="I29" t="s">
-        <v>43</v>
-      </c>
-      <c r="J29" s="1">
-        <v>45663.2521686467</v>
-      </c>
-      <c r="K29" t="s">
-        <v>13</v>
-      </c>
+    <row r="16" spans="8:8">
+      <c r="H16" s="1"/>
+    </row>
+    <row r="17" spans="8:8">
+      <c r="H17" s="1"/>
+    </row>
+    <row r="18" spans="8:8">
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="8:8">
+      <c r="H19" s="1"/>
+    </row>
+    <row r="20" spans="8:8">
+      <c r="H20" s="1"/>
+    </row>
+    <row r="21" spans="8:8">
+      <c r="H21" s="1"/>
+    </row>
+    <row r="22" spans="8:8">
+      <c r="H22" s="1"/>
+    </row>
+    <row r="23" spans="8:8">
+      <c r="H23" s="2"/>
+    </row>
+    <row r="24" spans="8:8">
+      <c r="H24" s="1"/>
+    </row>
+    <row r="25" spans="8:8">
+      <c r="H25" s="1"/>
+    </row>
+    <row r="26" spans="8:10">
+      <c r="H26" s="1"/>
+      <c r="I26"/>
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" spans="8:10">
+      <c r="H27" s="1"/>
+      <c r="I27"/>
+      <c r="J27" s="1"/>
+    </row>
+    <row r="28" spans="8:10">
+      <c r="H28" s="1"/>
+      <c r="I28"/>
+      <c r="J28" s="1"/>
+    </row>
+    <row r="29" spans="8:10">
+      <c r="H29" s="1"/>
+      <c r="I29"/>
+      <c r="J29" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>